<commit_message>
Update SQL - Retail Sales Analysis_utf .csv.xlsx
</commit_message>
<xml_diff>
--- a/SQL - Retail Sales Analysis_utf .csv.xlsx
+++ b/SQL - Retail Sales Analysis_utf .csv.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Faseeh\Desktop\SQL-Projects\SQL - Retail Sales Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2CF1AD4B-11EF-421F-969D-7AF1A6BE0013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{F6B48BF7-D528-4BD9-AA9B-BCC8B81DBEBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{831F1DAD-A926-44EE-BD5D-CB156B615740}"/>
   </bookViews>
   <sheets>
     <sheet name="SQL - Retail Sales Analysis_utf" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SQL - Retail Sales Analysis_utf'!$A$1:$K$1</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -932,6 +935,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{108F7FAC-43EA-452E-B579-13C246FBE723}">
   <dimension ref="A1:K2001"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -70903,6 +70918,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K1" xr:uid="{108F7FAC-43EA-452E-B579-13C246FBE723}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>